<commit_message>
vault backup: 2026-06-20 18:25:02
</commit_message>
<xml_diff>
--- a/BWL/Übung/Übungen/UE0806_Investitionsrechnung/BWL2T2_07_UE08_Vorlage2.xlsx
+++ b/BWL/Übung/Übungen/UE0806_Investitionsrechnung/BWL2T2_07_UE08_Vorlage2.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="2"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="UE 08.1" sheetId="1" state="visible" r:id="rId2"/>
@@ -73,7 +73,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="75">
   <si>
     <t>UE08.1</t>
   </si>
@@ -453,17 +453,64 @@
     <t xml:space="preserve">Jährlicher Cashflow</t>
   </si>
   <si>
+    <t>Nettobarwert</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Berücksichtigung Liquiditionserlös</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NBW + Liquiditionserlös</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Interpretation: Ohne Berücksichtigung des Liquiditionserlös lohnt sich die Investition nur bei 4% Zinsen.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ansonsten lohnt sich die Investition bei 4, 6, und 8% Zinsen, jedoch nicht bei 10 % Zinsen.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unterschied Nettobarwert und Barwert</t>
+  </si>
+  <si>
     <t>UE08.5</t>
+  </si>
+  <si>
+    <t>Liquidiationserlös</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cashflow Jahr 6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">// Cashflow + Liquiditionserlös</t>
+  </si>
+  <si>
+    <t>Effektivverzinsung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NBW (als Test)</t>
+  </si>
+  <si>
+    <t>b)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Variante 2 ist besser. Dadurch dass der interne Zinsfuß höher ist, ist der Gesamtgewinn höher.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Das ist vor allem deshalb so, weil die Cashflows bei Variante 2 eher in den ersten Jahren gemacht werden,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dadurch werden diese Cashflows weniger abgezinst.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="3">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="_-&quot;€&quot;\ * #,##0_-;\-&quot;€&quot;\ * #,##0_-;_-&quot;€&quot;\ * &quot;-&quot;_-;_-@_-"/>
     <numFmt numFmtId="165" formatCode="_-&quot;€&quot;\ * #,##0.00_-;\-&quot;€&quot;\ * #,##0.00_-;_-&quot;€&quot;\ * &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="166" formatCode="&quot;€&quot;\ #,##0"/>
+    <numFmt numFmtId="167" formatCode="_-* #,##0.00\ [$€-407]_-;\-* #,##0.00\ [$€-407]_-;_-* &quot;-&quot;??\ [$€-407]_-;_-@_-"/>
+    <numFmt numFmtId="168" formatCode="#,##0.00\ [$€-407]"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -564,7 +611,7 @@
     <xf fontId="0" fillId="2" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0"/>
     <xf fontId="0" fillId="3" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="26">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="1" fillId="4" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="164" xfId="0" applyNumberFormat="1"/>
@@ -580,9 +627,6 @@
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
       <protection hidden="0" locked="1"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
-      <protection hidden="0" locked="1"/>
-    </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="10" xfId="0" applyNumberFormat="1"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="1" xfId="0" applyNumberFormat="1"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="166" xfId="0" applyNumberFormat="1"/>
@@ -590,6 +634,14 @@
     <xf fontId="0" fillId="2" borderId="0" numFmtId="0" xfId="1" applyFill="1"/>
     <xf fontId="0" fillId="2" borderId="0" numFmtId="166" xfId="1" applyNumberFormat="1" applyFill="1"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="9" xfId="0" applyNumberFormat="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="9" xfId="0" applyNumberFormat="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="167" xfId="0" applyNumberFormat="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="168" xfId="0" applyNumberFormat="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="168" xfId="0" applyNumberFormat="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="168" xfId="0" applyNumberFormat="1">
+      <protection hidden="0" locked="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="20% - Accent1" xfId="1" builtinId="30"/>
@@ -639,7 +691,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <person displayName="Hinterholzer Stefan" id="{73A8AD53-9BED-515D-C891-AFD4EE022FEB}" userId="S::P20016@fhooe.at::6a077e09-2621-4617-a214-6a0ae6f4ad8b" providerId="AD"/>
+  <person displayName="Hinterholzer Stefan" id="{587C982B-B6E2-9832-FAD1-57275F39D970}" userId="S::P20016@fhooe.at::6a077e09-2621-4617-a214-6a0ae6f4ad8b" providerId="AD"/>
 </personList>
 </file>
 
@@ -1178,11 +1230,11 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="A4" dT="2025-05-27T07:35:55.71Z" personId="{73A8AD53-9BED-515D-C891-AFD4EE022FEB}" id="{FBADFD58-0062-460C-B478-BF0E1A561B1D}" done="0">
+  <threadedComment ref="A4" dT="2025-05-27T07:35:55.71Z" personId="{587C982B-B6E2-9832-FAD1-57275F39D970}" id="{FBADFD58-0062-460C-B478-BF0E1A561B1D}" done="0">
     <text xml:space="preserve">Sie heißen deshalb Erfolgszahlungen weil sie nicht nur zahlungswirksam sondern auch erfolgswirksam sind (d.h. sie verändern das Ergebnis - Gewinn oder Verlust)
 </text>
   </threadedComment>
-  <threadedComment ref="A9" dT="2025-05-27T07:35:55.71Z" personId="{73A8AD53-9BED-515D-C891-AFD4EE022FEB}" id="{9B535F7F-7001-6361-A1B5-D14391AC019A}" done="0">
+  <threadedComment ref="A9" dT="2025-05-27T07:35:55.71Z" personId="{587C982B-B6E2-9832-FAD1-57275F39D970}" id="{9B535F7F-7001-6361-A1B5-D14391AC019A}" done="0">
     <text xml:space="preserve">Sie heißen deshalb Erfolgszahlungen weil sie nicht nur zahlungswirksam sondern auch erfolgswirksam sind (d.h. sie verändern das Ergebnis - Gewinn oder Verlust)
 </text>
   </threadedComment>
@@ -1296,11 +1348,11 @@
         <v>11</v>
       </c>
       <c r="B12" s="2">
-        <f>B6+$B$4/$B$5</f>
+        <f t="shared" ref="B12:B15" si="0">B6+$B$4/$B$5</f>
         <v>25000</v>
       </c>
       <c r="C12" s="2">
-        <f>C6+$C$4/$C$5</f>
+        <f t="shared" ref="C12:C15" si="1">C6+$C$4/$C$5</f>
         <v>40000</v>
       </c>
     </row>
@@ -1309,11 +1361,11 @@
         <v>12</v>
       </c>
       <c r="B13" s="2">
-        <f>B7+$B$4/$B$5</f>
+        <f t="shared" si="0"/>
         <v>30000</v>
       </c>
       <c r="C13" s="2">
-        <f>C7+$C$4/$C$5</f>
+        <f t="shared" si="1"/>
         <v>35000</v>
       </c>
     </row>
@@ -1322,11 +1374,11 @@
         <v>13</v>
       </c>
       <c r="B14" s="2">
-        <f>B8+$B$4/$B$5</f>
+        <f t="shared" si="0"/>
         <v>35000</v>
       </c>
       <c r="C14" s="2">
-        <f>C8+$C$4/$C$5</f>
+        <f t="shared" si="1"/>
         <v>25000</v>
       </c>
     </row>
@@ -1335,11 +1387,11 @@
         <v>14</v>
       </c>
       <c r="B15" s="2">
-        <f>B9+$B$4/$B$5</f>
+        <f t="shared" si="0"/>
         <v>35000</v>
       </c>
       <c r="C15" s="2">
-        <f>C9+$C$4/$C$5</f>
+        <f t="shared" si="1"/>
         <v>25000</v>
       </c>
     </row>
@@ -1657,24 +1709,24 @@
       <c r="A8" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="B8" s="13" t="s">
+      <c r="B8" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="C8" s="13" t="s">
+      <c r="C8" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="D8" s="13" t="s">
+      <c r="D8" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="E8" s="13" t="s">
+      <c r="E8" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="F8" s="13" t="s">
+      <c r="F8" s="12" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="9" ht="14.25">
-      <c r="A9" s="13" t="s">
+      <c r="A9" s="12" t="s">
         <v>41</v>
       </c>
       <c r="B9" s="4">
@@ -1722,7 +1774,7 @@
       <c r="A11" t="s">
         <v>44</v>
       </c>
-      <c r="B11" s="14">
+      <c r="B11" s="13">
         <v>0.080000000000000002</v>
       </c>
     </row>
@@ -1730,23 +1782,23 @@
       <c r="A14" t="s">
         <v>45</v>
       </c>
-      <c r="B14" s="15">
+      <c r="B14" s="14">
         <f>B9/(1+$B$11)^B10</f>
         <v>23148.148148148146</v>
       </c>
-      <c r="C14" s="15">
+      <c r="C14" s="14">
         <f>C9/(1+$B$11)^C10</f>
         <v>21433.470507544578</v>
       </c>
-      <c r="D14" s="15">
+      <c r="D14" s="14">
         <f>D9/(1+$B$11)^D10</f>
         <v>27784.12843570593</v>
       </c>
-      <c r="E14" s="15">
+      <c r="E14" s="14">
         <f>E9/(1+$B$11)^E10</f>
         <v>25726.044847875863</v>
       </c>
-      <c r="F14" s="15">
+      <c r="F14" s="14">
         <f>F9/(1+$B$11)^F10</f>
         <v>6805.8319703375291</v>
       </c>
@@ -1755,7 +1807,7 @@
       <c r="A16" t="s">
         <v>46</v>
       </c>
-      <c r="B16" s="15">
+      <c r="B16" s="14">
         <f>SUM(B14:F14)</f>
         <v>104897.62390961206</v>
       </c>
@@ -1772,7 +1824,7 @@
       <c r="A18" t="s">
         <v>48</v>
       </c>
-      <c r="B18" s="15">
+      <c r="B18" s="14">
         <f>B16-B17</f>
         <v>4897.6239096120553</v>
       </c>
@@ -1798,9 +1850,10 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col bestFit="1" customWidth="1" min="1" max="1" width="16.88671875"/>
+    <col bestFit="1" customWidth="1" min="1" max="1" width="29.58203125"/>
+    <col bestFit="1" min="2" max="5" width="13.28125"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1812,83 +1865,162 @@
       <c r="A3" t="s">
         <v>47</v>
       </c>
-      <c r="B3" s="16">
+      <c r="B3" s="15">
         <v>200000</v>
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="16"/>
+      <c r="B4" s="15"/>
     </row>
     <row r="5" ht="15.6">
-      <c r="B5" s="17" t="s">
+      <c r="B5" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="C5" s="17" t="s">
+      <c r="C5" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="D5" s="17" t="s">
+      <c r="D5" s="16" t="s">
         <v>52</v>
       </c>
-      <c r="E5" s="17" t="s">
+      <c r="E5" s="16" t="s">
         <v>53</v>
       </c>
-      <c r="F5" s="17" t="s">
+      <c r="F5" s="16" t="s">
         <v>54</v>
       </c>
-      <c r="G5" s="17" t="s">
+      <c r="G5" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="H5" s="17" t="s">
+      <c r="H5" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="I5" s="17" t="s">
+      <c r="I5" s="16" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="18" t="s">
+      <c r="A6" s="17" t="s">
         <v>58</v>
       </c>
-      <c r="B6" s="19">
+      <c r="B6" s="18">
         <v>32000</v>
       </c>
-      <c r="C6" s="19">
+      <c r="C6" s="18">
         <v>32000</v>
       </c>
-      <c r="D6" s="19">
+      <c r="D6" s="18">
         <v>32000</v>
       </c>
-      <c r="E6" s="19">
+      <c r="E6" s="18">
         <v>32000</v>
       </c>
-      <c r="F6" s="19">
+      <c r="F6" s="18">
         <v>32000</v>
       </c>
-      <c r="G6" s="19">
+      <c r="G6" s="18">
         <v>32000</v>
       </c>
-      <c r="H6" s="19">
+      <c r="H6" s="18">
         <v>32000</v>
       </c>
-      <c r="I6" s="19">
+      <c r="I6" s="18">
         <v>32000</v>
       </c>
+      <c r="L6" s="15"/>
     </row>
     <row r="8">
       <c r="A8" t="s">
         <v>44</v>
       </c>
-      <c r="B8" s="20">
+      <c r="B8" s="19">
         <v>0.040000000000000001</v>
       </c>
       <c r="C8" s="20">
-        <v>0.059999999999999998</v>
-      </c>
-      <c r="D8" s="20">
+        <v>0.058299999999999998</v>
+      </c>
+      <c r="D8" s="19">
         <v>0.080000000000000002</v>
       </c>
-      <c r="E8" s="20">
+      <c r="E8" s="19">
         <v>0.10000000000000001</v>
+      </c>
+    </row>
+    <row r="10" ht="14.25">
+      <c r="A10" t="s">
+        <v>59</v>
+      </c>
+      <c r="B10" s="21">
+        <f>NPV(B8,$B$6:$I$6)</f>
+        <v>215447.83599841272</v>
+      </c>
+      <c r="C10" s="21">
+        <f>NPV(C8,$B$6:$I$6)</f>
+        <v>200057.30481711807</v>
+      </c>
+      <c r="D10" s="21">
+        <f>NPV(D8,$B$6:$I$6)</f>
+        <v>183892.44619920955</v>
+      </c>
+      <c r="E10" s="21">
+        <f>NPV(E8,$B$6:$I$6)</f>
+        <v>170717.63833288525</v>
+      </c>
+    </row>
+    <row r="11" ht="14.25">
+      <c r="A11" t="s">
+        <v>60</v>
+      </c>
+      <c r="B11" s="22">
+        <f>30000/(1+B8)^8</f>
+        <v>21920.706150059512</v>
+      </c>
+      <c r="C11" s="22">
+        <f>30000/(1+C8)^8</f>
+        <v>19065.617933589383</v>
+      </c>
+      <c r="D11" s="22">
+        <f>30000/(1+D8)^8</f>
+        <v>16208.066535059272</v>
+      </c>
+      <c r="E11" s="22">
+        <f>30000/(1+E8)^8</f>
+        <v>13995.221406291992</v>
+      </c>
+    </row>
+    <row r="12" ht="14.25">
+      <c r="A12" t="s">
+        <v>61</v>
+      </c>
+      <c r="B12" s="21">
+        <f>SUM(B10:B11)</f>
+        <v>237368.54214847222</v>
+      </c>
+      <c r="C12" s="21">
+        <f>SUM(C10:C11)</f>
+        <v>219122.92275070745</v>
+      </c>
+      <c r="D12" s="21">
+        <f>SUM(D10:D11)</f>
+        <v>200100.51273426882</v>
+      </c>
+      <c r="E12" s="21">
+        <f>SUM(E10:E11)</f>
+        <v>184712.85973917725</v>
+      </c>
+    </row>
+    <row r="14" ht="14.25">
+      <c r="B14" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="15" ht="14.25">
+      <c r="B15" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="19" ht="14.25">
+      <c r="B19" t="s">
+        <v>64</v>
       </c>
     </row>
   </sheetData>
@@ -1901,16 +2033,16 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="12.44140625"/>
+    <col customWidth="1" min="1" max="1" width="17.140625"/>
     <col customWidth="1" min="2" max="2" width="14"/>
-    <col customWidth="1" min="3" max="3" width="11.6640625"/>
+    <col customWidth="1" min="3" max="3" width="14.7109375"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
     </row>
     <row r="3">
@@ -1922,6 +2054,147 @@
       </c>
       <c r="C3" t="s">
         <v>3</v>
+      </c>
+    </row>
+    <row r="6" ht="14.25">
+      <c r="A6" t="s">
+        <v>66</v>
+      </c>
+      <c r="B6" s="23">
+        <v>5000</v>
+      </c>
+      <c r="C6" s="23">
+        <v>6000</v>
+      </c>
+    </row>
+    <row r="7" ht="14.25">
+      <c r="B7" s="23"/>
+      <c r="C7" s="23"/>
+    </row>
+    <row r="8" ht="14.25">
+      <c r="A8" t="s">
+        <v>47</v>
+      </c>
+      <c r="B8" s="23">
+        <v>-100000</v>
+      </c>
+      <c r="C8" s="23">
+        <v>-100000</v>
+      </c>
+    </row>
+    <row r="9" ht="14.25">
+      <c r="A9" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" s="23">
+        <v>20000</v>
+      </c>
+      <c r="C9" s="23">
+        <v>25000</v>
+      </c>
+    </row>
+    <row r="10" ht="14.25">
+      <c r="A10" s="24" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" s="23">
+        <v>20000</v>
+      </c>
+      <c r="C10" s="25">
+        <v>25000</v>
+      </c>
+    </row>
+    <row r="11" ht="14.25">
+      <c r="A11" s="24" t="s">
+        <v>13</v>
+      </c>
+      <c r="B11" s="25">
+        <v>20000</v>
+      </c>
+      <c r="C11" s="25">
+        <v>23000</v>
+      </c>
+    </row>
+    <row r="12" ht="14.25">
+      <c r="A12" s="24" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" s="25">
+        <v>25000</v>
+      </c>
+      <c r="C12" s="25">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="13" ht="14.25">
+      <c r="A13" s="24" t="s">
+        <v>15</v>
+      </c>
+      <c r="B13" s="25">
+        <v>25000</v>
+      </c>
+      <c r="C13" s="25">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="14" ht="14.25">
+      <c r="A14" s="24" t="s">
+        <v>67</v>
+      </c>
+      <c r="B14" s="25">
+        <f>25000+B6</f>
+        <v>30000</v>
+      </c>
+      <c r="C14" s="25">
+        <f>25000+C6</f>
+        <v>31000</v>
+      </c>
+      <c r="D14" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="17" ht="14.25">
+      <c r="A17" t="s">
+        <v>69</v>
+      </c>
+      <c r="B17" s="13">
+        <f>IRR(B8:B14)</f>
+        <v>0.097676574072629835</v>
+      </c>
+      <c r="C17" s="13">
+        <f>IRR(C8:C14)</f>
+        <v>0.11430471116801129</v>
+      </c>
+    </row>
+    <row r="21" ht="14.25">
+      <c r="A21" t="s">
+        <v>70</v>
+      </c>
+      <c r="B21">
+        <f>NPV(B17,B9:B14)</f>
+        <v>100000.00000000006</v>
+      </c>
+      <c r="C21">
+        <f>NPV(C17,C9:C14)</f>
+        <v>100000.00000000001</v>
+      </c>
+    </row>
+    <row r="24" ht="14.25">
+      <c r="A24" t="s">
+        <v>71</v>
+      </c>
+      <c r="B24" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="25" ht="14.25">
+      <c r="B25" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="26" ht="14.25">
+      <c r="B26" t="s">
+        <v>74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>